<commit_message>
procurement: add barcodes to seasonal container (all 10 SKUs)
Filled Баркод column: supplier Korean EAN (8809*) for the 3 SKUs where it's
known (Round Lab, Celimax x2), WB barcodes (2039*/2040*) from WB API
sales.json for the remaining 7.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XzNBEf4vaaEHRqeR8ZkfFA
</commit_message>
<xml_diff>
--- a/outputs/procurement/container_top10_seasonal_2026-06-30.xlsx
+++ b/outputs/procurement/container_top10_seasonal_2026-06-30.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,6 +35,10 @@
     <font>
       <i val="1"/>
       <color rgb="00C55A11"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="6">
@@ -91,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -103,6 +107,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -468,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X18"/>
+  <dimension ref="A1:X20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -792,7 +797,11 @@
           <t>ENOUGH - Collagen Moisture Essential Cream [50ml] N</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr"/>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>2040441089354</t>
+        </is>
+      </c>
       <c r="D5" s="4" t="n">
         <v>6360</v>
       </c>
@@ -948,7 +957,11 @@
           <t>Etude Baking Powder Crunch Pore Scrub</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr"/>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>2037596130970</t>
+        </is>
+      </c>
       <c r="D7" s="4" t="n">
         <v>5894</v>
       </c>
@@ -1024,7 +1037,11 @@
           <t>Manyo_Galac_Vita_Serum</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr"/>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>2039239495040</t>
+        </is>
+      </c>
       <c r="D8" s="4" t="n">
         <v>4092</v>
       </c>
@@ -1100,7 +1117,11 @@
           <t>Manyo_Complex_Ampoule</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr"/>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>2039239295145</t>
+        </is>
+      </c>
       <c r="D9" s="4" t="n">
         <v>2791</v>
       </c>
@@ -1176,7 +1197,11 @@
           <t>JMSOLUTION - Mask Pack Disney</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>2039610320817</t>
+        </is>
+      </c>
       <c r="D10" s="4" t="n">
         <v>1982</v>
       </c>
@@ -1252,7 +1277,11 @@
           <t>Enough 8 Peptide Full Cover Perfect Foundation 21 тон</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr"/>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>2038199518745</t>
+        </is>
+      </c>
       <c r="D11" s="4" t="n">
         <v>1575</v>
       </c>
@@ -1328,7 +1357,11 @@
           <t>MANYO BIFIDA INFUSION SHOT AMPOULE 1DX [50ml]</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr"/>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>2049478612030</t>
+        </is>
+      </c>
       <c r="D12" s="4" t="n">
         <v>397</v>
       </c>
@@ -1437,6 +1470,7 @@
         <v/>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
@@ -1459,10 +1493,18 @@
         <v/>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Учтена сезонность 2025 (пик дек ×2.1) + 2 магазина (×1.6). Оранжевые=оценка.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Баркод: 8809*=EAN поставщика (Корея), 2039*=баркод WB</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
procurement: recompute seasonality from full-year 2025 orders
Replaced revenue-based seasonality (2 files) with order-quantity seasonality
from all 12 monthly 2025 P&L files. Order-based Sep-Dec window is x0.97
(milder than the x1.21 revenue proxy); Dec x1.18 not x2.11. Per-SKU factors:
Round Lab x2.50, Manyo serums x2.07-2.11, Enough Collagen x0.76, 8 Peptide
x0.40. Container reloaded to 26t/117 768 units/61.4M₽, added a Сезонность
2025 sheet with monthly index.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XzNBEf4vaaEHRqeR8ZkfFA
</commit_message>
<xml_diff>
--- a/outputs/procurement/container_top10_seasonal_2026-06-30.xlsx
+++ b/outputs/procurement/container_top10_seasonal_2026-06-30.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Заказ предварительный" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Сезонность 2025" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,10 +36,6 @@
     <font>
       <i val="1"/>
       <color rgb="00C55A11"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <sz val="9"/>
     </font>
   </fonts>
   <fills count="6">
@@ -95,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -107,7 +104,6 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -473,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X20"/>
+  <dimension ref="A1:X18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -635,7 +631,7 @@
         </is>
       </c>
       <c r="D3" s="4" t="n">
-        <v>53519</v>
+        <v>53823</v>
       </c>
       <c r="E3" s="4" t="n">
         <v>6220</v>
@@ -699,7 +695,7 @@
       </c>
       <c r="W3" s="1" t="inlineStr">
         <is>
-          <t>Магазины (множитель)</t>
+          <t>Магазины ×</t>
         </is>
       </c>
       <c r="X3" s="2" t="n">
@@ -723,7 +719,7 @@
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>35603</v>
+        <v>36160</v>
       </c>
       <c r="E4" s="4" t="n">
         <v>10930</v>
@@ -803,7 +799,7 @@
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>6360</v>
+        <v>7417</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>2672</v>
@@ -869,37 +865,37 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CELIMAX</t>
+          <t>ETUDE</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>CELIMAX THE VITA-A RETINOL SHOT TIGHTENING SERUM [30ml]</t>
+          <t>Etude Baking Powder Crunch Pore Scrub</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>8809700320805</t>
+          <t>2037596130970</t>
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>5923</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>10130</v>
+        <v>5823</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>6030</v>
       </c>
       <c r="F6" s="4">
         <f>$J6*$G6*$E6</f>
         <v/>
       </c>
-      <c r="G6" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>0.018</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>5.8</v>
+      <c r="G6" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>12.5</v>
       </c>
       <c r="J6" s="4">
         <f>ROUNDUP($D6/$G6,0)</f>
@@ -949,37 +945,37 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>ETUDE</t>
+          <t>CELIMAX</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Etude Baking Powder Crunch Pore Scrub</t>
+          <t>CELIMAX THE VITA-A RETINOL SHOT TIGHTENING SERUM [30ml]</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>2037596130970</t>
+          <t>8809700320805</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>5894</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>6030</v>
+        <v>4837</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>10130</v>
       </c>
       <c r="F7" s="4">
         <f>$J7*$G7*$E7</f>
         <v/>
       </c>
-      <c r="G7" s="5" t="n">
-        <v>50</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>0.024</v>
-      </c>
-      <c r="I7" s="5" t="n">
-        <v>12.5</v>
+      <c r="G7" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>5.8</v>
       </c>
       <c r="J7" s="4">
         <f>ROUNDUP($D7/$G7,0)</f>
@@ -1043,7 +1039,7 @@
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>4092</v>
+        <v>4154</v>
       </c>
       <c r="E8" s="5" t="n">
         <v>11669</v>
@@ -1123,7 +1119,7 @@
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>2791</v>
+        <v>2818</v>
       </c>
       <c r="E9" s="5" t="n">
         <v>16371</v>
@@ -1203,7 +1199,7 @@
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>1982</v>
+        <v>1618</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>7793</v>
@@ -1283,7 +1279,7 @@
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>1575</v>
+        <v>501</v>
       </c>
       <c r="E11" s="5" t="n">
         <v>5393</v>
@@ -1363,7 +1359,7 @@
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>397</v>
+        <v>311</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>18173</v>
@@ -1470,11 +1466,10 @@
         <v/>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>Вес контейнера, т</t>
+          <t>Вес, т</t>
         </is>
       </c>
       <c r="D15">
@@ -1485,7 +1480,7 @@
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
-          <t>Заполнение, %</t>
+          <t>Заполнение %</t>
         </is>
       </c>
       <c r="D16">
@@ -1493,19 +1488,203 @@
         <v/>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Учтена сезонность 2025 (пик дек ×2.1) + 2 магазина (×1.6). Оранжевые=оценка.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>Баркод: 8809*=EAN поставщика (Корея), 2039*=баркод WB</t>
-        </is>
+          <t>Сезонность по ФАКТУ заказов 2025 (окно сен-дек ×0.97) + 2 магазина ×1.6. Оранж=оценка.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Месяц</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Заказы косметики, шт</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Индекс сезонности</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Янв</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>38646</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1.62</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Фев</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>22293</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Мар</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>27124</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1.14</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Апр</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>27490</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1.15</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Май</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>19552</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Июн</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>18960</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Июл</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>15646</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Авг</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>23965</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1.01</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Сен</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>17067</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Окт</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>22655</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Ноя</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>24334</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Дек</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>28098</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1.18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>